<commit_message>
Align course authorities and portal mappings
</commit_message>
<xml_diff>
--- a/Teacher Resources (Start Here)/09_STARLAB_Project_Approval_System_Package/STARLAB_Project_Approval_Tracker.xlsx
+++ b/Teacher Resources (Start Here)/09_STARLAB_Project_Approval_System_Package/STARLAB_Project_Approval_Tracker.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Start Here" sheetId="1" r:id="Rf67a3ba5d1af489f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Approval Tracker" sheetId="2" r:id="Rccafa9c0c3d14804"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Safety Ethics Flags" sheetId="3" r:id="R68e249f866e14ec2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Conference Log" sheetId="4" r:id="R696a298abe2242fe"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mentor Review" sheetId="5" r:id="R5912169e57d84a80"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dropdown Lists" sheetId="6" r:id="R717ab33247334e9a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Start Here" sheetId="1" r:id="Re225780a80524d37"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Approval Tracker" sheetId="2" r:id="R425132813b984e45"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Safety Ethics Flags" sheetId="3" r:id="Rf30a479c4dd84a5f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Conference Log" sheetId="4" r:id="R9d28d06997ed4f91"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mentor Review" sheetId="5" r:id="R21e04978f8224a8c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dropdown Lists" sheetId="6" r:id="Rc834cb8c798d48d3"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -29,13 +29,13 @@
     <x:font>
       <x:b/>
       <x:sz val="18"/>
-      <x:color rgb="FFFFFF"/>
+      <x:color rgb="FFFFFFFF"/>
       <x:name val="Carlito"/>
     </x:font>
     <x:font>
       <x:b/>
       <x:sz val="11"/>
-      <x:color rgb="FFFFFF"/>
+      <x:color rgb="FFFFFFFF"/>
       <x:name val="Carlito"/>
     </x:font>
   </x:fonts>
@@ -48,17 +48,17 @@
     </x:fill>
     <x:fill>
       <x:patternFill patternType="solid">
-        <x:fgColor rgb="000000"/>
+        <x:fgColor rgb="FF000000"/>
       </x:patternFill>
     </x:fill>
     <x:fill>
       <x:patternFill patternType="solid">
-        <x:fgColor rgb="ED1C24"/>
+        <x:fgColor rgb="FFED1C24"/>
       </x:patternFill>
     </x:fill>
     <x:fill>
       <x:patternFill patternType="solid">
-        <x:fgColor rgb="F3F4F6"/>
+        <x:fgColor rgb="FFF3F4F6"/>
       </x:patternFill>
     </x:fill>
   </x:fills>
@@ -66,112 +66,56 @@
     <x:border/>
     <x:border/>
     <x:border>
-      <x:right>
-        <x:color rgb="E5E7EB"/>
-      </x:right>
-      <x:bottom>
-        <x:color rgb="E5E7EB"/>
-      </x:bottom>
+      <x:right/>
+      <x:bottom/>
     </x:border>
     <x:border>
-      <x:left>
-        <x:color rgb="E5E7EB"/>
-      </x:left>
-      <x:bottom>
-        <x:color rgb="E5E7EB"/>
-      </x:bottom>
+      <x:left/>
+      <x:bottom/>
     </x:border>
     <x:border>
-      <x:right>
-        <x:color rgb="E5E7EB"/>
-      </x:right>
-      <x:top>
-        <x:color rgb="E5E7EB"/>
-      </x:top>
-      <x:bottom>
-        <x:color rgb="E5E7EB"/>
-      </x:bottom>
+      <x:right/>
+      <x:top/>
+      <x:bottom/>
     </x:border>
     <x:border>
-      <x:left>
-        <x:color rgb="E5E7EB"/>
-      </x:left>
-      <x:top>
-        <x:color rgb="E5E7EB"/>
-      </x:top>
-      <x:bottom>
-        <x:color rgb="E5E7EB"/>
-      </x:bottom>
+      <x:left/>
+      <x:top/>
+      <x:bottom/>
     </x:border>
     <x:border>
-      <x:right>
-        <x:color rgb="E5E7EB"/>
-      </x:right>
-      <x:top>
-        <x:color rgb="E5E7EB"/>
-      </x:top>
+      <x:right/>
+      <x:top/>
     </x:border>
     <x:border>
-      <x:left>
-        <x:color rgb="E5E7EB"/>
-      </x:left>
-      <x:top>
-        <x:color rgb="E5E7EB"/>
-      </x:top>
+      <x:left/>
+      <x:top/>
     </x:border>
     <x:border>
-      <x:right>
-        <x:color rgb="E5E7EB"/>
-      </x:right>
-      <x:bottom>
-        <x:color rgb="E5E7EB"/>
-      </x:bottom>
+      <x:right/>
+      <x:bottom/>
     </x:border>
     <x:border>
-      <x:left>
-        <x:color rgb="E5E7EB"/>
-      </x:left>
-      <x:bottom>
-        <x:color rgb="E5E7EB"/>
-      </x:bottom>
+      <x:left/>
+      <x:bottom/>
     </x:border>
     <x:border>
-      <x:right>
-        <x:color rgb="E5E7EB"/>
-      </x:right>
-      <x:top>
-        <x:color rgb="E5E7EB"/>
-      </x:top>
-      <x:bottom>
-        <x:color rgb="E5E7EB"/>
-      </x:bottom>
+      <x:right/>
+      <x:top/>
+      <x:bottom/>
     </x:border>
     <x:border>
-      <x:left>
-        <x:color rgb="E5E7EB"/>
-      </x:left>
-      <x:top>
-        <x:color rgb="E5E7EB"/>
-      </x:top>
-      <x:bottom>
-        <x:color rgb="E5E7EB"/>
-      </x:bottom>
+      <x:left/>
+      <x:top/>
+      <x:bottom/>
     </x:border>
     <x:border>
-      <x:right>
-        <x:color rgb="E5E7EB"/>
-      </x:right>
-      <x:top>
-        <x:color rgb="E5E7EB"/>
-      </x:top>
+      <x:right/>
+      <x:top/>
     </x:border>
     <x:border>
-      <x:left>
-        <x:color rgb="E5E7EB"/>
-      </x:left>
-      <x:top>
-        <x:color rgb="E5E7EB"/>
-      </x:top>
+      <x:left/>
+      <x:top/>
     </x:border>
   </x:borders>
   <x:cellStyleXfs count="1">
@@ -285,78 +229,78 @@
   <x:dxfs count="11">
     <x:dxf>
       <x:fill>
-        <x:patternFill patternType="solid">
-          <x:bgColor rgb="FEE2E2"/>
+        <x:patternFill>
+          <x:bgColor rgb="FFFEE2E2"/>
         </x:patternFill>
       </x:fill>
     </x:dxf>
     <x:dxf>
       <x:fill>
-        <x:patternFill patternType="solid">
-          <x:bgColor rgb="FEF3C7"/>
+        <x:patternFill>
+          <x:bgColor rgb="FFFEF3C7"/>
         </x:patternFill>
       </x:fill>
     </x:dxf>
     <x:dxf>
       <x:fill>
-        <x:patternFill patternType="solid">
-          <x:bgColor rgb="DCFCE7"/>
+        <x:patternFill>
+          <x:bgColor rgb="FFDCFCE7"/>
         </x:patternFill>
       </x:fill>
     </x:dxf>
     <x:dxf>
       <x:fill>
-        <x:patternFill patternType="solid">
-          <x:bgColor rgb="FEE2E2"/>
+        <x:patternFill>
+          <x:bgColor rgb="FFFEE2E2"/>
         </x:patternFill>
       </x:fill>
     </x:dxf>
     <x:dxf>
       <x:fill>
-        <x:patternFill patternType="solid">
-          <x:bgColor rgb="FEF3C7"/>
+        <x:patternFill>
+          <x:bgColor rgb="FFFEF3C7"/>
         </x:patternFill>
       </x:fill>
     </x:dxf>
     <x:dxf>
       <x:fill>
-        <x:patternFill patternType="solid">
-          <x:bgColor rgb="DCFCE7"/>
+        <x:patternFill>
+          <x:bgColor rgb="FFDCFCE7"/>
         </x:patternFill>
       </x:fill>
     </x:dxf>
     <x:dxf>
       <x:fill>
-        <x:patternFill patternType="solid">
-          <x:bgColor rgb="FEE2E2"/>
+        <x:patternFill>
+          <x:bgColor rgb="FFFEE2E2"/>
         </x:patternFill>
       </x:fill>
     </x:dxf>
     <x:dxf>
       <x:fill>
-        <x:patternFill patternType="solid">
-          <x:bgColor rgb="FEE2E2"/>
+        <x:patternFill>
+          <x:bgColor rgb="FFFEE2E2"/>
         </x:patternFill>
       </x:fill>
     </x:dxf>
     <x:dxf>
       <x:fill>
-        <x:patternFill patternType="solid">
-          <x:bgColor rgb="FEF3C7"/>
+        <x:patternFill>
+          <x:bgColor rgb="FFFEF3C7"/>
         </x:patternFill>
       </x:fill>
     </x:dxf>
     <x:dxf>
       <x:fill>
-        <x:patternFill patternType="solid">
-          <x:bgColor rgb="FEF3C7"/>
+        <x:patternFill>
+          <x:bgColor rgb="FFFEF3C7"/>
         </x:patternFill>
       </x:fill>
     </x:dxf>
     <x:dxf>
       <x:fill>
-        <x:patternFill patternType="solid">
-          <x:bgColor rgb="FEE2E2"/>
+        <x:patternFill>
+          <x:bgColor rgb="FFFEE2E2"/>
         </x:patternFill>
       </x:fill>
     </x:dxf>
@@ -495,9 +439,9 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Calibri"/>
-        <a:ea typeface="Calibri"/>
-        <a:cs typeface="Calibri"/>
+        <a:latin typeface="Calibri Light"/>
+        <a:ea typeface="Calibri Light"/>
+        <a:cs typeface="Calibri Light"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -619,7 +563,7 @@
     </x:row>
     <x:row r="4">
       <x:c r="A4" s="12" t="str">
-        <x:v>Use this workbook to track student project approval status, safety and ethics flags, conference notes, mentor review, and next actions. Update it after every approval conference, method revision, project pivot, or safety/ethics review.</x:v>
+        <x:v>Use this workbook as the official record of project approval status. Its Dropdown Lists approval statuses are authoritative. Update it after every approval conference, method revision, project pivot, safety/ethics review, or decision to begin systematic data collection.</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
@@ -649,7 +593,7 @@
       </x:c>
       <x:c r="E9" s="32" t="n">
         <x:f>COUNTA('Approval Tracker'!A2:A51)</x:f>
-        <x:v>50</x:v>
+        <x:v>0</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
@@ -675,7 +619,7 @@
         <x:v>Running record of teacher-student conferences and approval decisions.</x:v>
       </x:c>
       <x:c r="D11" s="33" t="str">
-        <x:v>Approved for Data Collection</x:v>
+        <x:v>Approved for Systematic Data Collection</x:v>
       </x:c>
       <x:c r="E11" s="34" t="n">
         <x:f>COUNTIF('Approval Tracker'!E2:E51,"Approved for Systematic Data Collection")</x:f>
@@ -705,7 +649,7 @@
         <x:v>Protected reference lists for data validation options.</x:v>
       </x:c>
       <x:c r="D13" s="33" t="str">
-        <x:v>Needs Safety/Ethics Review</x:v>
+        <x:v>Needs Safety or Ethics Review</x:v>
       </x:c>
       <x:c r="E13" s="34" t="n">
         <x:f>COUNTIF('Approval Tracker'!E2:E51,"Needs Safety Review")+COUNTIF('Approval Tracker'!E2:E51,"Needs Ethics Review")</x:f>
@@ -732,7 +676,7 @@
         <x:v>Local Policy</x:v>
       </x:c>
       <x:c r="B15" s="12" t="str">
-        <x:v>This tracker supports but does not replace district safety policies or required approval forms.</x:v>
+        <x:v>This tracker supports district policy. The district supplies any required safety, consent, media, fieldwork, equipment, chemical, drone, privacy, human-participant, IRB/SRC, or related forms.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -4196,7 +4140,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rce83fe7c73e84307"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfed9b4ad0f8b4e2d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7681,7 +7625,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rde008ac90cea4305"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rffb61f385a054269"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -11096,7 +11040,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6924c3d9beb84c8f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0b3807f75f46494e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -14527,7 +14471,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7671abba4e884323"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd5e3d770a6814a0a"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>